<commit_message>
feat: add Flutter integration test suite task (IMP-012) to improvements tracker
- Added IMP-012 to tasks/generate_improvements.py covering 6 critical user flows
- Regenerated tasks/vela_improvements.xlsx (now 12 improvements)
- Flutter mobile session detail modal, timeline, progress fixes
- Agent and CLAUDE.md doc updates
- Android manifest, issue tracker, and manifest-coach agent additions

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issues/master_issue_tracker.xlsx
+++ b/issues/master_issue_tracker.xlsx
@@ -613,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V38"/>
+  <dimension ref="A1:V42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4589,6 +4589,402 @@
           <t>Duplicate of CU-008 which shows resolved — needs re-verification</t>
         </is>
       </c>
+    </row>
+    <row r="39" ht="60" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>UI-12</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Sessions Not Loading on Timeline Screen</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Mobile</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Manual Testing</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Investigator Agent</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Flutter App</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>vela_flutter/lib/data/repositories/progress_repository.dart, vela_flutter/lib/providers/progress_provider.dart</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Investigator Agent</t>
+        </is>
+      </c>
+      <c r="Q39" s="2" t="inlineStr">
+        <is>
+          <t>Sessions tab permanently shows loading/error state and never displays sessions. getSessions() called ApiConstants.sessions (/progress/sessions) — a route that does not exist in the backend. Even if the URL were correct, response.data was cast directly as List, but the real endpoint GET /api/progress/:subject_id returns { sessions: [...], topics: [...], revisionItems: [...], pagination: {...} } — sessions is a nested key, not the root value. getTopics() had the same two bugs (/progress/topics + response.data as List). The provider called three separate Future.wait requests all hitting the same endpoint, tripling network traffic.</t>
+        </is>
+      </c>
+      <c r="R39" s="2" t="inlineStr">
+        <is>
+          <t>Added getProgress(subjectId) method to ProgressRepository that calls GET /api/progress/:subjectId and returns the full Map. getSessions() and getTopics() now delegate to getProgress() and extract response.data['sessions'] and response.data['topics'] respectively. ProgressNotifier.loadProgress() refactored to call getProgress() once and unpack sessions + topics from a single network response.</t>
+        </is>
+      </c>
+      <c r="S39" s="2" t="inlineStr">
+        <is>
+          <t>Open Sessions tab with an active subject — sessions list should render. Open network inspector and confirm exactly one GET /api/progress/:id request fires on load (not three). Pull-to-refresh and re-open — list reloads correctly.</t>
+        </is>
+      </c>
+      <c r="T39" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="U39" s="2" t="inlineStr"/>
+      <c r="V39" s="2" t="inlineStr">
+        <is>
+          <t>Backend endpoint GET /api/progress/:subject_id does NOT use the standard { data: [], pagination: {} } envelope — it uses top-level keys. This is the only progress endpoint that exists for subject-scoped data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="60" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>UI-13</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Session cards not tappable — no detail view</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Mobile</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Interaction Completeness Audit</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Investigator Agent</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Flutter App</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>vela_flutter/lib/ui/screens/sessions/session_detail_modal.dart (new), vela_flutter/lib/ui/screens/sessions/timeline_screen.dart</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Investigator Agent</t>
+        </is>
+      </c>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t>Tapping a session card on the Timeline screen did nothing. _SessionCard had onEdit and onDelete callbacks but no onTap for a detail view. Users expect tapping a card to open its detail — the missing interaction was identified by the Step 3 Interaction Completeness Audit.</t>
+        </is>
+      </c>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>Created SessionDetailModal (modelled on TaskDetailModal) showing activity type, date, duration, topics, full notes, URL/YouTube thumbnail, revision badge, and Edit/Delete actions with confirmation dialog. Added onTap prop to _SessionCard, wrapped VelaCard in GestureDetector, added _showSessionDetail() to _TimelineScreenState, and wired onTap in the SliverList builder.</t>
+        </is>
+      </c>
+      <c r="S40" s="2" t="inlineStr">
+        <is>
+          <t>Tap a session card on the Timeline screen — SessionDetailModal opens with full session info. Tap Edit — modal closes and AddSessionModal opens pre-filled. Tap Delete — confirmation dialog appears; confirm closes modal and removes session. Slidable swipe-to-delete and inline Edit/Delete buttons still work independently.</t>
+        </is>
+      </c>
+      <c r="T40" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="U40" s="2" t="inlineStr"/>
+      <c r="V40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="60" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>UI-14</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Session goal badge missing; attachment stub misleading</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Mobile</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Web Parity Review</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Investigator Agent</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Flutter App</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>vela_flutter/lib/ui/screens/sessions/session_detail_modal.dart, vela_flutter/lib/ui/screens/sessions/timeline_screen.dart</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr"/>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Investigator Agent</t>
+        </is>
+      </c>
+      <c r="Q41" s="2" t="inlineStr">
+        <is>
+          <t>Web parity review against Timeline.jsx found two gaps. (1) When a session has a goal_id, the web card shows a teal goal badge with the linked goal title. Neither _SessionCard nor SessionDetailModal showed this — users had no way to see which goal a session contributed to. (2) SessionDetailModal's Attachments section showed an 'Add Attachment' button that fired showSnackBar('coming soon') — actively misleading users into thinking they could add attachments when the feature is not implemented.</t>
+        </is>
+      </c>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t>Fix 1 — Goal badge in SessionDetailModal: converted StatelessWidget to ConsumerWidget, resolved goalTitle via ref.watch(goalsProvider), and added a VelaBadgeVariant.success badge (flag icon + truncated title, max 140px) after the revision badge in the meta Wrap, guarded by if (goalTitle != null). Fix 2 — Attachment stub removal: replaced the OutlinedButton/snackbar with a read-only display — muted 'No attachments' text when count is 0, or a VelaBadge with paperclip icon and count when attachments exist. Fix 3 — Goal badge on _SessionCard: added optional goalTitle String? prop, resolved at SliverList build time via ref.watch(goalsProvider) (keeps _SessionCard a plain StatelessWidget), and rendered a success badge after the revision badge in the activity type row.</t>
+        </is>
+      </c>
+      <c r="S41" s="2" t="inlineStr">
+        <is>
+          <t>Create a session linked to a goal. Open the Sessions tab — _SessionCard should show a green flag badge with the goal title next to the revision badge. Tap the card — SessionDetailModal should show the same badge in the meta row. Open a session with no goal — no badge appears. Open the modal for a session with 0 attachments — 'No attachments' muted text appears instead of the Add Attachment button. For a session with attachments the count badge renders. No snackbar fires in either case.</t>
+        </is>
+      </c>
+      <c r="T41" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="U41" s="2" t="inlineStr"/>
+      <c r="V41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42" ht="60" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>UI-15</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>SessionDetailModal 'Add Attachment' button fires no feedback</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Mobile</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Task — Fix non-functional button</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Investigator Agent</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Flutter App</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>vela_flutter/lib/ui/screens/sessions/session_detail_modal.dart</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr"/>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Investigator Agent</t>
+        </is>
+      </c>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t>The '+ Add Attachment' button in SessionDetailModal had an empty onPressed: () { // TODO } lambda. Tapping it produced zero visual feedback — no snackbar, no navigation, no modal. Web parity check confirmed Timeline.jsx has no equivalent button at all (attachment_count is display-only). Backend progress.js has no writable endpoint for session-attachment linking. The feature does not exist on any platform, so the button was silently swallowing taps.</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>Replaced the empty onPressed lambda with a ScaffoldMessenger snackbar ('Attachment linking for sessions is coming soon.', 2-second duration). The button remains visible so users know the feature is planned, but every tap now produces visible feedback. No API calls, no navigation.</t>
+        </is>
+      </c>
+      <c r="S42" s="2" t="inlineStr">
+        <is>
+          <t>Open any session detail modal. Tap '+ Add Attachment'. A snackbar should appear at the bottom of the screen with the 'coming soon' message and dismiss after 2 seconds. No crash, no silent swallow.</t>
+        </is>
+      </c>
+      <c r="T42" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="U42" s="2" t="inlineStr"/>
+      <c r="V42" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
@@ -7576,7 +7972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V16"/>
+  <dimension ref="A1:V20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7606,7 +8002,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>Flutter Mobile  —  14 issue(s)</t>
+          <t>Flutter Mobile  —  18 issue(s)</t>
         </is>
       </c>
     </row>
@@ -9125,6 +9521,402 @@
         </is>
       </c>
       <c r="V16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>UI-12</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Sessions Not Loading on Timeline Screen</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Mobile</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Manual Testing</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Investigator Agent</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Flutter App</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>vela_flutter/lib/data/repositories/progress_repository.dart, vela_flutter/lib/providers/progress_provider.dart</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Investigator Agent</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>Sessions tab permanently shows loading/error state and never displays sessions. getSessions() called ApiConstants.sessions (/progress/sessions) — a route that does not exist in the backend. Even if the URL were correct, response.data was cast directly as List, but the real endpoint GET /api/progress/:subject_id returns { sessions: [...], topics: [...], revisionItems: [...], pagination: {...} } — sessions is a nested key, not the root value. getTopics() had the same two bugs (/progress/topics + response.data as List). The provider called three separate Future.wait requests all hitting the same endpoint, tripling network traffic.</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>Added getProgress(subjectId) method to ProgressRepository that calls GET /api/progress/:subjectId and returns the full Map. getSessions() and getTopics() now delegate to getProgress() and extract response.data['sessions'] and response.data['topics'] respectively. ProgressNotifier.loadProgress() refactored to call getProgress() once and unpack sessions + topics from a single network response.</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="inlineStr">
+        <is>
+          <t>Open Sessions tab with an active subject — sessions list should render. Open network inspector and confirm exactly one GET /api/progress/:id request fires on load (not three). Pull-to-refresh and re-open — list reloads correctly.</t>
+        </is>
+      </c>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="U17" s="2" t="inlineStr"/>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>Backend endpoint GET /api/progress/:subject_id does NOT use the standard { data: [], pagination: {} } envelope — it uses top-level keys. This is the only progress endpoint that exists for subject-scoped data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>UI-13</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Session cards not tappable — no detail view</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Mobile</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Interaction Completeness Audit</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Investigator Agent</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Flutter App</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>vela_flutter/lib/ui/screens/sessions/session_detail_modal.dart (new), vela_flutter/lib/ui/screens/sessions/timeline_screen.dart</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Investigator Agent</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>Tapping a session card on the Timeline screen did nothing. _SessionCard had onEdit and onDelete callbacks but no onTap for a detail view. Users expect tapping a card to open its detail — the missing interaction was identified by the Step 3 Interaction Completeness Audit.</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>Created SessionDetailModal (modelled on TaskDetailModal) showing activity type, date, duration, topics, full notes, URL/YouTube thumbnail, revision badge, and Edit/Delete actions with confirmation dialog. Added onTap prop to _SessionCard, wrapped VelaCard in GestureDetector, added _showSessionDetail() to _TimelineScreenState, and wired onTap in the SliverList builder.</t>
+        </is>
+      </c>
+      <c r="S18" s="2" t="inlineStr">
+        <is>
+          <t>Tap a session card on the Timeline screen — SessionDetailModal opens with full session info. Tap Edit — modal closes and AddSessionModal opens pre-filled. Tap Delete — confirmation dialog appears; confirm closes modal and removes session. Slidable swipe-to-delete and inline Edit/Delete buttons still work independently.</t>
+        </is>
+      </c>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr"/>
+      <c r="V18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>UI-14</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Session goal badge missing; attachment stub misleading</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Mobile</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Web Parity Review</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Investigator Agent</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Flutter App</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>vela_flutter/lib/ui/screens/sessions/session_detail_modal.dart, vela_flutter/lib/ui/screens/sessions/timeline_screen.dart</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Investigator Agent</t>
+        </is>
+      </c>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>Web parity review against Timeline.jsx found two gaps. (1) When a session has a goal_id, the web card shows a teal goal badge with the linked goal title. Neither _SessionCard nor SessionDetailModal showed this — users had no way to see which goal a session contributed to. (2) SessionDetailModal's Attachments section showed an 'Add Attachment' button that fired showSnackBar('coming soon') — actively misleading users into thinking they could add attachments when the feature is not implemented.</t>
+        </is>
+      </c>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>Fix 1 — Goal badge in SessionDetailModal: converted StatelessWidget to ConsumerWidget, resolved goalTitle via ref.watch(goalsProvider), and added a VelaBadgeVariant.success badge (flag icon + truncated title, max 140px) after the revision badge in the meta Wrap, guarded by if (goalTitle != null). Fix 2 — Attachment stub removal: replaced the OutlinedButton/snackbar with a read-only display — muted 'No attachments' text when count is 0, or a VelaBadge with paperclip icon and count when attachments exist. Fix 3 — Goal badge on _SessionCard: added optional goalTitle String? prop, resolved at SliverList build time via ref.watch(goalsProvider) (keeps _SessionCard a plain StatelessWidget), and rendered a success badge after the revision badge in the activity type row.</t>
+        </is>
+      </c>
+      <c r="S19" s="2" t="inlineStr">
+        <is>
+          <t>Create a session linked to a goal. Open the Sessions tab — _SessionCard should show a green flag badge with the goal title next to the revision badge. Tap the card — SessionDetailModal should show the same badge in the meta row. Open a session with no goal — no badge appears. Open the modal for a session with 0 attachments — 'No attachments' muted text appears instead of the Add Attachment button. For a session with attachments the count badge renders. No snackbar fires in either case.</t>
+        </is>
+      </c>
+      <c r="T19" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="U19" s="2" t="inlineStr"/>
+      <c r="V19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>UI-15</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>SessionDetailModal 'Add Attachment' button fires no feedback</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Mobile</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Task — Fix non-functional button</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Investigator Agent</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Flutter App</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>vela_flutter/lib/ui/screens/sessions/session_detail_modal.dart</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Investigator Agent</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>The '+ Add Attachment' button in SessionDetailModal had an empty onPressed: () { // TODO } lambda. Tapping it produced zero visual feedback — no snackbar, no navigation, no modal. Web parity check confirmed Timeline.jsx has no equivalent button at all (attachment_count is display-only). Backend progress.js has no writable endpoint for session-attachment linking. The feature does not exist on any platform, so the button was silently swallowing taps.</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>Replaced the empty onPressed lambda with a ScaffoldMessenger snackbar ('Attachment linking for sessions is coming soon.', 2-second duration). The button remains visible so users know the feature is planned, but every tap now produces visible feedback. No API calls, no navigation.</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>Open any session detail modal. Tap '+ Add Attachment'. A snackbar should appear at the bottom of the screen with the 'coming soon' message and dismiss after 2 seconds. No crash, no silent swallow.</t>
+        </is>
+      </c>
+      <c r="T20" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="U20" s="2" t="inlineStr"/>
+      <c r="V20" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:V2"/>
@@ -10335,7 +11127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -10357,7 +11149,7 @@
         </is>
       </c>
       <c r="B2" s="23" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
@@ -10367,7 +11159,7 @@
         </is>
       </c>
       <c r="B3" s="25" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
@@ -10416,7 +11208,7 @@
         </is>
       </c>
       <c r="B9" s="23" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -10433,7 +11225,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
@@ -10443,7 +11235,7 @@
         </is>
       </c>
       <c r="B13" s="29" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
@@ -10453,7 +11245,7 @@
         </is>
       </c>
       <c r="B14" s="31" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -10463,7 +11255,7 @@
         </is>
       </c>
       <c r="B15" s="33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
@@ -10490,7 +11282,7 @@
         </is>
       </c>
       <c r="B19" s="23" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
@@ -10543,37 +11335,47 @@
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="22" t="inlineStr">
         <is>
+          <t>Flutter Investigator Agent</t>
+        </is>
+      </c>
+      <c r="B26" s="23" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
           <t>User</t>
         </is>
       </c>
-      <c r="B26" s="23" t="n">
+      <c r="B27" s="23" t="n">
         <v>22</v>
       </c>
     </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="21" t="inlineStr">
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="21" t="inlineStr">
         <is>
           <t>Open Issues by Priority</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="30" t="inlineStr">
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="30" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="B29" s="31" t="n">
+      <c r="B30" s="31" t="n">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A28:C28"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A29:C29"/>
     <mergeCell ref="A7:C7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>